<commit_message>
[Data] json 데이터 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Skill.xlsx
+++ b/JsonConverter/ExcelFiles/Skill.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\오즈_과제\UnityMiniProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40BA9291-23C6-4375-9858-7E873A027954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF15DD06-CAE7-45DE-B8AE-1162637CDAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36765" yWindow="1125" windowWidth="15450" windowHeight="14175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36765" yWindow="1125" windowWidth="18570" windowHeight="14175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId1"/>
@@ -101,11 +101,11 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>KNOCKBACK:2,DAMAGE:2</t>
+    <t>DAMAGE:1,SELFHEAL:3</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>DAMAGE:1,SELFHEAL:3</t>
+    <t>DASHSLASH:3:5</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -576,7 +576,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -607,7 +607,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>

</xml_diff>